<commit_message>
atualizado o status dos fluxos e pendencias
</commit_message>
<xml_diff>
--- a/conteudo/Sprint_Review_Controle_Entregas.xlsx
+++ b/conteudo/Sprint_Review_Controle_Entregas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Resumo da Sprint" sheetId="1" state="visible" r:id="rId3"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="292">
   <si>
     <t xml:space="preserve">RESUMO GERAL DAS SPRINTS — SISTEMA DE GESTÃO DE CONTRATOS</t>
   </si>
@@ -490,9 +490,6 @@
     <t xml:space="preserve">Teste automatizado funcionalidade de Segmentação</t>
   </si>
   <si>
-    <t xml:space="preserve">A fazer</t>
-  </si>
-  <si>
     <t xml:space="preserve">BackEnd referente a funcionalidade Configurações Gerais</t>
   </si>
   <si>
@@ -502,6 +499,9 @@
     <t xml:space="preserve">Desenvolvimento da CRUD(Create Configurações Gerais, Ready Configurações Gerais, Update Configurações Gerais, Delete Configurações Gerais) referente a funcionalidade em questão.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fazendo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Analise geral do acesso ao Snow Flake</t>
   </si>
   <si>
@@ -772,58 +772,61 @@
     <t xml:space="preserve">oportunidade-em-andamento.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Aprovado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluxo New Name.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-name.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-base-cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Base (Cliente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluxo de nova base de cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-base-cliente.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-base-produto-ou-modulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Base (Produto ou Módulo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluxo de nova base de produto ou módulo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new-base-produto-ou-modulo.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">complementacao-do-contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complementação do Contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluxo de complementação de dados do contrato.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">complementacao-do-contrato.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aguardando aprovação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fluxo New Name.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-name.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-base-cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Base (Cliente)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fluxo de nova base de cliente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-base-cliente.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-base-produto-ou-modulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Base (Produto ou Módulo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fluxo de nova base de produto ou módulo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new-base-produto-ou-modulo.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">complementacao-do-contrato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complementação do Contrato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fluxo de complementação de dados do contrato.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">complementacao-do-contrato.png</t>
   </si>
   <si>
     <t xml:space="preserve">validacao-oportunidades-renovacao</t>
@@ -3147,7 +3150,7 @@
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>154</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3158,7 +3161,7 @@
         <v>2043</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>45</v>
@@ -3167,7 +3170,7 @@
         <v>42</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>154</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3178,16 +3181,16 @@
         <v>2044</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="E15" s="1" t="s">
         <v>42</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>154</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3207,7 +3210,7 @@
         <v>148</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="73.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3465,7 +3468,7 @@
         <v>46290</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>172</v>
@@ -3530,6 +3533,9 @@
   </sheetPr>
   <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.44"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
@@ -3650,9 +3656,12 @@
       <c r="B10" s="1" t="n">
         <v>10</v>
       </c>
+      <c r="C10" s="0" t="n">
+        <v>9</v>
+      </c>
       <c r="D10" s="1" t="n">
         <f aca="false">D9+C10</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3664,7 +3673,7 @@
       </c>
       <c r="D11" s="1" t="n">
         <f aca="false">D10+C11</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3676,7 +3685,7 @@
       </c>
       <c r="D12" s="1" t="n">
         <f aca="false">D11+C12</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3688,7 +3697,7 @@
       </c>
       <c r="D13" s="1" t="n">
         <f aca="false">D12+C13</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3700,7 +3709,7 @@
       </c>
       <c r="D14" s="1" t="n">
         <f aca="false">D13+C14</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3712,7 +3721,7 @@
       </c>
       <c r="D15" s="1" t="n">
         <f aca="false">D14+C15</f>
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -4105,7 +4114,7 @@
         <v>265</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>249</v>
@@ -4116,19 +4125,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>266</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>248</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>249</v>
@@ -4139,19 +4148,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4159,19 +4168,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="24" t="s">
+        <v>273</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>273</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>273</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G12" s="14" t="s">
         <v>272</v>
-      </c>
-      <c r="C12" s="24" t="s">
-        <v>272</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>272</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4179,19 +4188,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4199,19 +4208,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>249</v>
@@ -4222,19 +4231,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>249</v>
@@ -4245,19 +4254,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>249</v>
@@ -4268,19 +4277,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>